<commit_message>
Major changes for DOC, PRO and Sections
</commit_message>
<xml_diff>
--- a/uploads/PRO-01-B.xlsx
+++ b/uploads/PRO-01-B.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijasoka/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijasoka/Downloads/3. PROCEDIMIENTOS ESPECIFICOS Y OBLIGATORIOS/PRO-01 Procedimiento para mejora continua/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5D8658-15E6-F24A-AAD9-3BAF6CF2DA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9765635-843A-914C-86D0-29754957700C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -675,9 +675,9 @@
   <cols>
     <col min="1" max="1" width="2.6640625" style="6" customWidth="1"/>
     <col min="2" max="2" width="10.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34" style="6" customWidth="1"/>
-    <col min="4" max="4" width="27.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="33.83203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="40.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.5" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.33203125" style="6" bestFit="1" customWidth="1"/>

</xml_diff>